<commit_message>
feat(camera): add verified desktop tactical controls
- add fixed-pitch tactical camera with bounded zoom
- add playable battle-grid camera bounds
- add screen-relative keyboard and right-drag panning
- add 45-degree snapped Q/E rotation
- prevent battlefield input through visible HUD panels
- add Studio-only camera recovery test controls
- preserve mobile gesture UAT as pending
- defer Focus Selected integration to Slice 7 View Mode
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Game_Rules.xlsx
+++ b/docs/CTRBLXAI_Game_Rules.xlsx
@@ -19768,7 +19768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D53"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20897,7 +20897,6 @@
         </is>
       </c>
     </row>
-    <row r="53"/>
   </sheetData>
   <autoFilter ref="A1:D49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -37836,7 +37835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F46"/>
+  <dimension ref="A1:F47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -39226,6 +39225,38 @@
       <c r="F46" t="inlineStr">
         <is>
           <t>All main stats -10%. Does not stack with itself.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Statuses Buff</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Guard</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Buff (Dispellable)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>1 turn (until next ready turn)</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Refresh duration</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Reduces incoming final damage by 35% (base). Guard Bonus passives add to mitigation (e.g., Shield +15%). Total capped at 80%. Dispellable by Purge/Dispel. Removed by hard CC (Stun, Freeze, Sleep). Guard RT = round(Modified Base RT × 0.10) + 50% Effective Armor Off-Hand WT. 2H weapon → Off-Hand WT = 0. Once per turn, 1 AP.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: Implement StyleBootstrap for dynamic UI styling with tokens, themes, and design rules
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Game_Rules.xlsx
+++ b/docs/CTRBLXAI_Game_Rules.xlsx
@@ -35,6 +35,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Terrain Effects" sheetId="26" state="visible" r:id="rId26"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Objects Encounters" sheetId="27" state="visible" r:id="rId27"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Open Decisions" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Persistent HP MP" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01 Project Identity'!$A$1:$D$79</definedName>
@@ -36522,6 +36523,693 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>PERSISTENT HP/MP AND RECOVERY RULES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Post-battle recovery, KO handling, MP regen, base behavior, deployment, and Max HP/MP change rules.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Source: CTRBLXAI.db persistent_hp_mp_rules (25 rows)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>topic</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>rule</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Persistent Resources</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Battle Start</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Battle Start HP = Persistent Current HP. Battle Start MP = Persistent Current MP. Starting a battle does not refill either resource.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Persistent Resources</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>New Unit Init</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Newly created or recruited units initialize at full HP and full MP once. Not a recurring battle-start rule.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Recovery Formula</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>After every qualifying completed battle, each surviving owned unit recovers: HP Recovery = ceil(Max HP × 0.35), MP Recovery = ceil(Max MP × 0.35). Current = min(Max, Current + Recovery).</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>35% is working value; verify through expedition testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Deployed and Benched</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Recovery applies to ALL surviving owned units whether deployed or benched. A unit at 0% would reach full after ~3 qualifying battles.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Qualifying Battle</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Recovery triggers only when encounter completes legitimate victory requirements and runs normal completion processing. Abandoned, cancelled, failed-to-init, dev-test, or zero-completion do not grant recovery.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Timing</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Victory met → finish current action + triggered resolutions → persist final HP/MP/Item charges → apply post-battle recovery → end battle.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Post-Battle Recovery</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>No Free Phase</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Once victory requirements satisfied, battle ends after active resolution chain. Players cannot continue casting, using Items, regenerating, or repositioning. Use recovery Skills BEFORE the finishing action.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>KO Rules</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>KO Penalty</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>KO units receive NO post-battle HP or MP recovery. Remain KO until roster returns to base.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KO Rules</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Base Clears KO</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Returning to base clears KO first during base processing. Unit receives Current HP = 1. Current MP unchanged (stays at whatever it was at KO). Returning to base does NOT otherwise restore HP or MP.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Locked. 1 HP is intentionally harsh — unit needs recovery battles or healing Items before being combat-ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>10</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>KO Rules</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Design Intent</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>KO is materially worse than surviving at low HP without requiring permanent injury or death.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Natural MP Regen</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>MP Regen = 2 + floor(INT / 40) MP per 1000 CT. Base 2 ensures all units regenerate naturally. Every 40 INT adds +1. No cap. Accumulator += CT Passed × MP Regen / 1000. When Accumulator ≥ 1: restore floor(Accumulator) MP, retain fraction.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Coefficient 6 is working value; test against Skill MP costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Natural MP Regen</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Properties</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Visible Derived Stat. Linear formula: base 2 + floor(INT/40). Based on elapsed CT (not ready turns) so fast units do not regenerate more. No cap. Intentionally provides baseline recovery to all units while rewarding INT investment at clear breakpoints.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Natural MP Regen</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Reference Table</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>INT 0=2, INT 40=3, INT 80=4, INT 120=5, INT 160=6, INT 200=7, INT 240=8, INT 300=9 MP per 1000 CT.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>14</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Natural MP Regen</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Timing</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Only progresses while battle CT is advancing. Does not progress while paused, disconnected, loading, or waiting in decision menu where CT is stopped.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>15</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Recovery Stalling</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Policy</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>No cap on natural MP regen, no reward for fast victories, no penalty for long battles. Deliberate stalling is allowed — elapsed time, AP, RT, MP costs, and Item charges are accepted opportunity costs.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>16</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Recovery Stalling</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Safety</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Instant or zero-time resource-positive loops remain invalid. A repeatable effect must not restore more MP than it spends without elapsed CT, a finite charge, a sacrifice, or another real resource.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>17</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Base Rules</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Items at Base</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Items cannot be used at base. Returning to base replenishes all charged Item uses. Because Items cannot be activated at base, charge replenishment cannot convert into unlimited HP/MP recovery.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>18</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Base Rules</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Base Does Not Heal</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Returning to base does NOT restore HP or MP. Only clears KO and replenishes Item charges.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>19</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Max Resource Changes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Max Increases</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>If Maximum increases: Current Resource += New Maximum − Old Maximum. Preserves amount missing.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Max Resource Changes</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Max Decreases</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>If Maximum decreases: Current Resource = min(Current Resource, New Maximum). Clamps without conversion.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>21</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Passive Interactions</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Arcane Flow</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Remains explicit ready-turn MP recovery passive (not CT-based). Does not become part of MP Regen stat. Value may need retest after persistent MP implemented.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>22</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Passive Interactions</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Sleep</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Intentionally both hard control AND expedition recovery tool. Sleeping units recover HP/MP per Sleep rule. Allowing enemy to stay asleep also lets enemy recover — tactical risk.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>23</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Passive Interactions</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Quiver Quick Draw</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Retains 10% Max MP activation payment as working value. Persistent MP makes this more consequential. Adjust only after playtesting.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Working</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Deployment UI</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Resource Readiness</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Deployment interface must expose: Current HP/Max HP, Current MP/Max MP, Item charges, KO status. Warn when team has low HP, low MP, depleted Items, or KO members. Warning informs but does not block deployment.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>25</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Starter Support</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Starting Items</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Starting units receive existing Small Healing Potions and Ether Cell. No tutorial-only consumable. Early tutorial should demonstrate Item use + base charge replenishment.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add AffixData module for item affix name lookup
- Introduced a new Lua module `AffixData.lua` that contains a structured lookup for item affix names categorized into numerical and passive types.
- The numerical affixes include various bonuses and resistances with corresponding tiers.
- The passive affixes include unique effects identified by their IDs.
- This module is auto-generated from the database and should not be manually edited.
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Game_Rules.xlsx
+++ b/docs/CTRBLXAI_Game_Rules.xlsx
@@ -37,6 +37,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="18 Open Decisions" sheetId="28" state="visible" r:id="rId28"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="19 Persistent HP MP" sheetId="29" state="visible" r:id="rId29"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 Item Affix Names" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21 Unit Progression" sheetId="31" state="visible" r:id="rId31"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'01 Project Identity'!$A$1:$D$79</definedName>
@@ -42054,6 +42055,664 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>UNIT XP AND LEVELING SYSTEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Completion XP + procedural objective bonuses. Objectives generated from encounter content, not authored per encounter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>XP Model</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Completion + Procedural Objective Bonus. Base XP per battle completion, bonus XP from procedurally generated objectives derived from encounter content.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>XP Model</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Fell Seal (objective bonuses) + Crawl Tactics (procedural encounters) hybrid. Objectives are NOT authored per encounter — they are generated from spawned content.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Award timing</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>XP awarded after battle completion. All deployed units receive base XP. Benched units receive 50%.</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Base formula</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Base XP = Encounter Base XP × Level Scaling Factor</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Locked direction — exact values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Level Scaling Factor</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Diminishing returns when unit level exceeds encounter level. Bonus when underleveled. Exact formula pending.</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Encounter Base XP</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Authored per encounter type: normal, elite, boss, quest. Exact values pending.</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Anti-farming</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Trivial content provides sharply reduced XP. Same direction as Guild XP anti-farming rule.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Human passive</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Human Adaptability: EXP gained +10%. Applied to total XP (base + bonuses).</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Locked — references races table</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Benched units</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Deployed units receive 100% XP. Benched owned units receive 50%. Prevents permanent roster gaps.</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Base XP</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>KO units</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>KO'd units still receive XP if battle is won. They participated.</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Level Curve</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>XP to next level = floor(100 × Level^1.4). Exact exponent and base pending simulation.</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Level Curve</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Reference values</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>L1→2: 100 XP. L10→11: ~2,512 XP. L50→51: ~36,840 XP. L99 cap.</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Working baseline — pending simulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Level Curve</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Level cap</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>99. No XP earned past cap.</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Level Curve</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Stat gain on level-up</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Base stats recalculated from race growth rates: baseStat = startingStat + floor(growthRate × (level - 1)). Already implemented in RaceData.CalcBaseStats.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Locked — already functional</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Objectives are generated from encounter content at battle start, not authored per encounter. Each spawned feature may create an objective.</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Objective sources</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Objectives derive from what the encounter generator placed: elite enemies, NPCs, map objects, terrain features, spawn timing, enemy composition.</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Bonus range</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Each objective grants 10-50% bonus XP on top of base. Multiple objectives may be active. All are optional.</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Locked direction — exact values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Player visibility</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Active objectives shown at battle start and during battle. Completion shown in real-time. Final summary at battle end.</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>No penalty</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Failing an objective grants zero bonus — never reduces base XP. Objectives are purely additive.</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Elite enemy spawned</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Defeat the elite enemy within N turns. Bonus: 25-40%.</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Example — values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>NPC spawned</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Protect the NPC — NPC survives the battle. Bonus: 20-30%.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Example — values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Siege object spawned</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Hit N enemies with the ballista/catapult. Bonus: 15-25%.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Example — values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Speed objective</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Win within N turns. Turn count scales with encounter size. Bonus: 15-25%.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Example — always available</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Flawless objective</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>No unit KO'd. Bonus: 20-30%.</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Example — always available</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>All defeated</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Defeat all enemies (not just win condition). Bonus: 10-15%.</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Example — always available</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Functional owner</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Slice 6 owns XP system design and implementation. Unit Level already exists as a field. RaceData.CalcBaseStats already recalculates stats from level.</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Dependencies</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Slice 5 (procedural maps) must exist before procedural objectives can detect spawned content. Base XP (completion only) can work without Slice 5.</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Guild XP relationship</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Unit XP and Guild XP are separate systems. Guild XP is account-wide progression. Unit XP is per-unit stat progression. Both award after battle completion.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Add simulation report for CTRBLXAI XP System on 2026-09-12
- Documented formulas and validation against database reference values
- Analyzed level curve pacing across tiers and identified pacing issues
- Evaluated effectiveness of overleveled penalties and underleveled bonuses
- Assessed enemy composition XP ranges and their impact on gameplay
- Compared human passive XP advantage against non-human units
- Investigated benched unit gap and its implications for roster management
- Provided critical action items for XP system adjustments
</commit_message>
<xml_diff>
--- a/docs/CTRBLXAI_Game_Rules.xlsx
+++ b/docs/CTRBLXAI_Game_Rules.xlsx
@@ -42061,7 +42061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42074,7 +42074,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Completion XP + procedural objective bonuses. Objectives generated from encounter content, not authored per encounter.</t>
+          <t>Kill-based XP + procedural objectives. Linear ramp: XP to level = 500 + (Level × 20). L99 cap at launch. Evolutions post-launch.</t>
         </is>
       </c>
     </row>
@@ -42113,12 +42113,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Completion + Procedural Objective Bonus. Base XP per battle completion, bonus XP from procedurally generated objectives derived from encounter content.</t>
+          <t>Completion + Procedural Objective Bonus. Base XP per enemy killed, scaling with enemy level. Bonus XP from procedurally generated objectives. Quest board shows biome, rewards, and XP range upfront. XP requirement grows with level — early levels fast, later levels slower.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
@@ -42130,12 +42130,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Reference</t>
+          <t>XP per kill</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Fell Seal (objective bonuses) + Crawl Tactics (procedural encounters) hybrid. Objectives are NOT authored per encounter — they are generated from spawned content.</t>
+          <t>Kill XP = Base Type XP × (1 + Enemy Level / 50). Higher level enemies give more XP.</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -42147,281 +42147,281 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>XP Model</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Award timing</t>
+          <t>Quest display</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>XP awarded after battle completion. All deployed units receive base XP. Benched units receive 50%.</t>
+          <t>Quest board shows: biome, quest type, recommended level, enemy count range, reward drops, gold, and XP range (min-max based on enemies defeated).</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Locked direction</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Enemy Base XP</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Base formula</t>
+          <t>Grunt</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Base XP = Encounter Base XP × Level Scaling Factor</t>
+          <t>20 XP base. Standard filler enemy.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Locked direction — exact values pending</t>
+          <t>Working baseline</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Enemy Base XP</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Level Scaling Factor</t>
+          <t>Veteran</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Diminishing returns when unit level exceeds encounter level. Bonus when underleveled. Exact formula pending.</t>
+          <t>35 XP base. Tier 1+ standard, Tier 0 rare.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Working baseline</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Enemy Base XP</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Encounter Base XP</t>
+          <t>Elite</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Authored per encounter type: normal, elite, boss, quest. Exact values pending.</t>
+          <t>60 XP base. 1-2 per quest when present.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Working baseline</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Enemy Base XP</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Anti-farming</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Trivial content provides sharply reduced XP. Same direction as Guild XP anti-farming rule.</t>
+          <t>120 XP base. Quest objective, usually 1.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Working baseline</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Human passive</t>
+          <t>Grunt L1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Human Adaptability: EXP gained +10%. Applied to total XP (base + bonuses).</t>
+          <t>20 × (1 + 1/50) = 20 XP</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Locked — references races table</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Benched units</t>
+          <t>Grunt L50</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Deployed units receive 100% XP. Benched owned units receive 50%. Prevents permanent roster gaps.</t>
+          <t>20 × (1 + 50/50) = 40 XP</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Base XP</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>KO units</t>
+          <t>Grunt L99</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>KO'd units still receive XP if battle is won. They participated.</t>
+          <t>20 × (1 + 99/50) = 60 XP</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Level Curve</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Formula</t>
+          <t>Grunt L150</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>XP to next level = floor(100 × Level^1.4). Exact exponent and base pending simulation.</t>
+          <t>20 × (1 + 150/50) = 80 XP</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Working baseline</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Level Curve</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Reference values</t>
+          <t>Grunt L250</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>L1→2: 100 XP. L10→11: ~2,512 XP. L50→51: ~36,840 XP. L99 cap.</t>
+          <t>20 × (1 + 250/50) = 120 XP</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Working baseline — pending simulation</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Level Curve</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Level cap</t>
+          <t>Elite L99</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>99. No XP earned past cap.</t>
+          <t>60 × (1 + 99/50) = 179 XP</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Locked</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Level Curve</t>
+          <t>Kill XP Scaling</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Stat gain on level-up</t>
+          <t>Boss L200</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Base stats recalculated from race growth rates: baseStat = startingStat + floor(growthRate × (level - 1)). Already implemented in RaceData.CalcBaseStats.</t>
+          <t>120 × (1 + 200/50) = 600 XP</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Locked — already functional</t>
+          <t>Reference</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Evolution Tiers</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>System</t>
+          <t>Future tiers</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Objectives are generated from encounter content at battle start, not authored per encounter. Each spawned feature may create an objective.</t>
+          <t>Additional evolution tiers extend by adding one XP/level value. Clean extension.</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -42433,83 +42433,83 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Level Curve</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Objective sources</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Objectives derive from what the encounter generator placed: elite enemies, NPCs, map objects, terrain features, spawn timing, enemy composition.</t>
+          <t>Linear ramp: XP to next level = 500 + (Level × 20). Higher levels require more XP. This counteracts enemy-level kill scaling to produce natural pacing: early levels ~4 battles, late levels ~6-7 battles.</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Level Curve</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Bonus range</t>
+          <t>Level cap</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Each objective grants 10-50% bonus XP on top of base. Multiple objectives may be active. All are optional.</t>
+          <t>99 at launch. Racial evolutions (extending to 199, 299) are post-launch features. Tier 1 and Tier 2 XP formulas will be set when evolutions release, informed by live player data.</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Locked direction — exact values pending</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Level Curve</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Player visibility</t>
+          <t>Stat gain</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Active objectives shown at battle start and during battle. Completion shown in real-time. Final summary at battle end.</t>
+          <t>Base stats recalculated from race growth rates: baseStat = startingStat + floor(growthRate × (level - 1)). Already implemented in RaceData.CalcBaseStats.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Locked direction</t>
+          <t>Locked — already functional</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>XP Distribution</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>No penalty</t>
+          <t>Battle formula</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Failing an objective grants zero bonus — never reduces base XP. Objectives are purely additive.</t>
+          <t>Battle XP = sum of (Base Type XP × (1 + Enemy Level / 50)) for each enemy defeated. Plus objective bonuses.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -42521,190 +42521,850 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>XP Distribution</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Elite enemy spawned</t>
+          <t>Deployed units</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Defeat the elite enemy within N turns. Bonus: 25-40%.</t>
+          <t>100% of battle XP.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Example — values pending</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>XP Distribution</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>NPC spawned</t>
+          <t>Benched units</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Protect the NPC — NPC survives the battle. Bonus: 20-30%.</t>
+          <t>50% of battle XP. Prevents permanent roster gaps.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Example — values pending</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>XP Distribution</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Siege object spawned</t>
+          <t>KO'd units</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hit N enemies with the ballista/catapult. Bonus: 15-25%.</t>
+          <t>Receive full XP if battle is won. They participated.</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Example — values pending</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>XP Distribution</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Speed objective</t>
+          <t>Human passive</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Win within N turns. Turn count scales with encounter size. Bonus: 15-25%.</t>
+          <t>Adaptability: total XP (kills + objectives) × 1.10.</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Example — always available</t>
+          <t>Locked — references races table</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Level Scaling</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Flawless objective</t>
+          <t>On-level (gap ≤5)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>No unit KO'd. Bonus: 20-30%.</t>
+          <t>×1.0 — no penalty.</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Example — always available</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Procedural Objectives</t>
+          <t>Level Scaling</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>All defeated</t>
+          <t>Gap 6-10</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Defeat all enemies (not just win condition). Bonus: 10-15%.</t>
+          <t>×0.75</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Example — always available</t>
+          <t>Locked</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ownership</t>
+          <t>Level Scaling</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Functional owner</t>
+          <t>Gap 11-15</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Slice 6 owns XP system design and implementation. Unit Level already exists as a field. RaceData.CalcBaseStats already recalculates stats from level.</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>×0.50</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ownership</t>
+          <t>Level Scaling</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Dependencies</t>
+          <t>Gap 16-20</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Slice 5 (procedural maps) must exist before procedural objectives can detect spawned content. Base XP (completion only) can work without Slice 5.</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr"/>
+          <t>×0.25</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>Level Scaling</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Gap 21+</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>×0.10 — trivial content.</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Level Scaling</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Underleveled ≤-5</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>×1.25</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Level Scaling</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Underleveled ≤-10</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>×1.50 (cap)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Level Scaling</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Level Gap = Unit Level - Quest Recommended Level. Multiplier applied to all kill XP.</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Generated from encounter content at battle start. Not authored per encounter. Each spawned feature may create an objective. All optional — failure never reduces base XP.</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Elite spawned</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Defeat the elite within N turns. Bonus: 25-40% of base XP.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>NPC spawned</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>NPC survives the battle. Bonus: 20-30%.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Siege object</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Hit N enemies with ballista/catapult. Bonus: 15-25%.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Speed clear</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Win within N turns (scales with encounter size). Bonus: 15-25%. Always available.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Flawless</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>No unit KO'd. Bonus: 20-30%. Always available.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Procedural Objectives</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>All defeated</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Defeat all enemies (not just win condition). Bonus: 10-15%. Always available.</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Working baseline</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Normal battle</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Standard combat encounter. XP from kills.</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Elite battle</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Contains elite enemies. Higher XP per kill.</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Boss battle</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Contains boss enemy. Highest per-kill XP.</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Slay X</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Defeat X specific enemies. Kill count determines XP.</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Survive</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Survive N turns. Minimum XP guaranteed on completion. Enemies defeated add additional XP.</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Protect</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Protect NPC/object. Minimum XP guaranteed. Enemies defeated add additional XP.</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Quest Types</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Exploration</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Series of battles. Each battle awards XP separately. Total = sum of individual battles.</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>System</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Dispatched units earn flat XP based on dispatch difficulty × duration. Unit unavailable for N battles.</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Dispatch</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>XP formula</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dispatch XP = Dispatch Difficulty XP × Duration Multiplier. Roughly equivalent to one battle's kills as tradeoff for no player control.</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Locked direction — exact values pending</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Anti-Farming</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Rule</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Trivial content provides sharply reduced XP via overleveled penalty. Same direction as Guild XP anti-farming.</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>Ownership</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Functional owner</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Slice 6 owns XP system implementation. Base formula can work without Slice 5. Procedural objectives need Slice 5 map spawns.</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Dependencies</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Slice 5: procedural maps for objectives. Slice 8: quest board, dispatch, exploration. Daily/seasonal events: separate reward systems, may grant XP as part of reward.</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Ownership</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
         <is>
           <t>Guild XP relationship</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Unit XP and Guild XP are separate systems. Guild XP is account-wide progression. Unit XP is per-unit stat progression. Both award after battle completion.</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Unit XP and Guild XP are separate. Guild XP = account progression (merchants, facilities). Unit XP = per-unit stat progression. Both award after battle. Separate formulas.</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
         <is>
           <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Platform Features</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Seasonal events</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Top players can become random boss encounters. Limited-time Unique rarity items. Special event XP sources possible.</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Locked direction — Roblox live-service features</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Platform Features</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Daily events</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Special resources (e.g., item level-up materials). May include XP bonuses.</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Platform Features</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Progression breadth</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Leveling is one of many parallel systems: Guild Level, equipment rarity, loadout customization, quest variety, exploration, dispatch, seasonal events, daily events. Level cap is a long-term milestone, not the only goal.</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Level Curve</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>XP to next level = 500 + (Level × 20). L1→2: 520 XP. L10→11: 700 XP. L25→26: 1,000 XP. L50→51: 1,500 XP. L75→76: 2,000 XP. L98→99: 2,460 XP.</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Evolution Tiers</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Launch (Tier 0)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Level 1-99. XP to next level = 500 + (Level × 20). No evolutions at launch. Total XP L1→99: ~145,000 XP.</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Evolution Tiers</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Post-launch evolutions</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1st Evolution (L100-199): unlocks Skill Slot 5, improved racial perk/drawback. 2nd Evolution (L200-299): unlocks 2nd Doctrine slot, further improved racials. XP formulas for Tier 1 and 2 set at release using live data.</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Evolution Tiers</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Future tiers</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Additional evolution tiers extend level cap. Formula calibrated from live data at each release.</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Locked direction</t>
         </is>
       </c>
     </row>

</xml_diff>